<commit_message>
Small adjustment to competency Excel-file
</commit_message>
<xml_diff>
--- a/data/source/Kompetanse_Anonymisert.xlsx
+++ b/data/source/Kompetanse_Anonymisert.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://helsemidtno-my.sharepoint.com/personal/jo_willy_grawe_stolav_no/Documents/Dokumenter/Prosjekter og langsiktig/Automatisk rullering (ressursstyring og planlegging)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://helsemidtno-my.sharepoint.com/personal/jo_willy_grawe_stolav_no/Documents/VSCode/Rullering/Planlegger/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="116" documentId="11_F25DC773A252ABDACC104859B15D4E1E5ADE58F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CDDB306-562F-42ED-8FBB-69A4D31F95C5}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="11_F25DC773A252ABDACC104859B15D4E1E5ADE58F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B53A9A96-6741-49CF-A5B4-C2781F754048}"/>
   <bookViews>
-    <workbookView xWindow="33204" yWindow="612" windowWidth="27288" windowHeight="15168" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1740" yWindow="1188" windowWidth="27600" windowHeight="14244" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -84,12 +84,6 @@
     <t>Navn på ansatt</t>
   </si>
   <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>Employee 1</t>
   </si>
   <si>
@@ -295,6 +289,12 @@
   </si>
   <si>
     <t>Employee 69</t>
+  </si>
+  <si>
+    <t>Ja</t>
+  </si>
+  <si>
+    <t>Ukjent</t>
   </si>
 </sst>
 </file>
@@ -360,17 +360,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -384,7 +391,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FA91C1EF-DE32-4969-9D83-FDB97A1B764A}" name="Tabell1" displayName="Tabell1" ref="A2:O71" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FA91C1EF-DE32-4969-9D83-FDB97A1B764A}" name="Kompetanseoversikt" displayName="Kompetanseoversikt" ref="A2:O71" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A2:O71" xr:uid="{FA91C1EF-DE32-4969-9D83-FDB97A1B764A}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{6F968E1D-9BD4-417C-8578-7926C76BCD4E}" name="Navn på ansatt"/>
@@ -673,8 +680,8 @@
   <dimension ref="A1:O71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.109375" customWidth="1"/>
-    <col min="2" max="2" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.88671875" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" customWidth="1"/>
     <col min="3" max="3" width="25.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.77734375" customWidth="1"/>
@@ -734,1251 +741,1251 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:15" s="5" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G3" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I4" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M4" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N4" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O4" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I6" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K6" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H7" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I7" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J7" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K7" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M7" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G8" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H8" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I8" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K8" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H9" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I9" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K9" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M9" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N9" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H10" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I10" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K10" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M10" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N10" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O10" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H12" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I12" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J12" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I13" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M13" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N13" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H14" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G15" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H15" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I15" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J15" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K15" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G16" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H16" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I16" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J16" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K16" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G17" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H17" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I17" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J17" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K17" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H18" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I18" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J18" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K18" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O19" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I20" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J20" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="K20" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N20" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H21" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I21" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J21" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K21" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M21" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N21" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O21" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B22" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H22" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I22" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G23" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H23" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I23" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J23" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K23" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B24" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G24" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H24" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I24" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J24" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K24" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B25" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G25" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H25" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I25" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J25" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K25" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B26" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G26" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H26" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I26" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J26" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K26" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B27" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H27" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K27" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M27" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B28" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H28" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I28" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J28" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K28" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="M29" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N29" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O29" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M30" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N30" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O30" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B31" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G31" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H31" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I31" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J31" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K31" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="M31" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N31" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O31" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B32" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G32" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H32" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I32" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J32" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K32" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M32" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B33" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H33" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I33" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J33" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M33" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N33" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O33" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B34" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G34" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H34" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I34" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J34" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M34" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B35" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I35" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K35" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B36" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G36" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H36" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I36" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J36" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M36" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B37" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G37" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H37" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I37" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J37" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K37" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B38" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I38" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K38" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B39" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G39" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H39" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I39" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J39" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K39" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B40" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G40" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H40" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I40" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J40" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K40" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="O41" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B42" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I42" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K42" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B43" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H43" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I43" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J43" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B44" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="G44" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H44" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I44" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J44" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K44" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B45" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I45" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B46" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I46" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B47" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I47" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B48" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I48" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K48" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B49" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I49" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K49" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B50" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I50" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K50" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B51" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I51" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K51" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B52" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I52" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B53" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I53" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K53" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B54" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I54" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K54" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B55" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I55" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B56" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I56" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B57" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B58" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I58" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B59" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I59" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B60" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I60" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B61" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I61" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K61" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="K62" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K63" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="M63" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="N63" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="K64" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K65" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B66" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I66" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="K66" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K67" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I68" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B69" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I69" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I70" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J70" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B71" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H71" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="I71" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J71" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>